<commit_message>
Update Approaches for S-104 in different countries.xlsx
Based on feedback after TWCWG10 and presentations during the meeting
</commit_message>
<xml_diff>
--- a/S-104/HOs different approaches/Approaches for S-104 in different countries.xlsx
+++ b/S-104/HOs different approaches/Approaches for S-104 in different countries.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kartverket-my.sharepoint.com/personal/hilde_sande_borck_kartverket_no/Documents/TWCWG/arbeid/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kartverket-my.sharepoint.com/personal/hilde_sande_borck_kartverket_no/Documents/repos/TWCWG/S-104/HOs different approaches/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{124C2C49-7D91-4E8D-B6A0-64371711F684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F985ECB-6F1F-4D69-9477-00CD16B80F74}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{22976B59-201B-4FEA-BD03-99E4E46465BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4976DF68-907B-46F3-94D4-2E5C8E2172EA}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="1650" windowWidth="28545" windowHeight="17850" xr2:uid="{C4867061-5DD6-4A1F-ABA3-31C353E062FB}"/>
+    <workbookView xWindow="2910" yWindow="1110" windowWidth="33540" windowHeight="18705" xr2:uid="{C4867061-5DD6-4A1F-ABA3-31C353E062FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="37">
   <si>
     <t>Predicted tide</t>
   </si>
@@ -103,6 +103,51 @@
   </si>
   <si>
     <t>Norway</t>
+  </si>
+  <si>
+    <t>New Zealand</t>
+  </si>
+  <si>
+    <t>jcoppola@linz.govt.nz</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>anni.jokiniemi@fmi.fi</t>
+  </si>
+  <si>
+    <t>E-mail</t>
+  </si>
+  <si>
+    <t>Hilde Sande Borck</t>
+  </si>
+  <si>
+    <t>Anni Jokiniemi</t>
+  </si>
+  <si>
+    <t>Jennifer Coppola</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>(Edited by Hilde SB based on TWCWG10 presentation)</t>
+  </si>
+  <si>
+    <t>Andreas Boesch</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>Trials</t>
+  </si>
+  <si>
+    <t>Zarina Jayaswal</t>
+  </si>
+  <si>
+    <t>USA</t>
   </si>
 </sst>
 </file>
@@ -184,10 +229,11 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A471F449-EDF7-4F88-AA84-F1B36EC5E416}" name="Tabell3" displayName="Tabell3" ref="G1:G1048576" totalsRowShown="0">
-  <autoFilter ref="G1:G1048576" xr:uid="{A471F449-EDF7-4F88-AA84-F1B36EC5E416}"/>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{96BBCB90-8256-43A3-85DD-5CDD7B515FC5}" name="Main contact"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A471F449-EDF7-4F88-AA84-F1B36EC5E416}" name="Tabell3" displayName="Tabell3" ref="G1:H1048576" totalsRowShown="0">
+  <autoFilter ref="G1:H1048576" xr:uid="{A471F449-EDF7-4F88-AA84-F1B36EC5E416}"/>
+  <tableColumns count="2">
+    <tableColumn id="2" xr3:uid="{ACBDCDFF-10EF-4168-BB4F-0227374F6E24}" name="Main contact"/>
+    <tableColumn id="1" xr3:uid="{96BBCB90-8256-43A3-85DD-5CDD7B515FC5}" name="E-mail"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -522,18 +568,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06659A35-34AF-4A2C-9D69-F422D682FD8E}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.140625" customWidth="1"/>
     <col min="3" max="3" width="103.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="68.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.140625" customWidth="1"/>
     <col min="6" max="6" width="45.5703125" customWidth="1"/>
-    <col min="7" max="7" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" customWidth="1"/>
+    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -555,8 +602,11 @@
       <c r="G1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -572,18 +622,130 @@
       <c r="E2" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" xr:uid="{920CD4AD-62F1-4C2E-9E8F-C18B3FE15CD9}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{920CD4AD-62F1-4C2E-9E8F-C18B3FE15CD9}"/>
+    <hyperlink ref="H3" r:id="rId2" xr:uid="{93E7D7D2-0AA3-412B-B872-8A3466A6D954}"/>
+    <hyperlink ref="H4" r:id="rId3" xr:uid="{3D3EE3DB-2192-424F-BCB3-4538F70D294A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED</oddFooter>
+  </headerFooter>
   <tableParts count="2">
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -621,7 +783,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31955A9E-0217-4F67-8A40-6C933139A431}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="103.140625" bestFit="1" customWidth="1"/>
@@ -687,6 +849,10 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;12&amp;K000000 UNCLASSIFIED</oddFooter>
+  </headerFooter>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>